<commit_message>
added NED data, updated cost calculations, RG results
</commit_message>
<xml_diff>
--- a/market_clearing/economic_summary.xlsx
+++ b/market_clearing/economic_summary.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10513"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipenoris/tmp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/laura_linuesa-domenech_tennet_eu/Documents/Thesis/Code/market_clearing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C353BCB8-5EC8-0143-BDD3-A1B661DAACD7}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="115_{DB14EC48-4273-41AA-9C67-5EBA85351DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="460" windowWidth="28040" windowHeight="17040" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" r:id="rId4" sheetId="2"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,9 +26,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
-  <si>
-    <t>ECONOMIC SUMMARY (30 days simulation)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+  <si>
+    <t>ECONOMIC SUMMARY (31 days simulation)</t>
   </si>
   <si>
     <t>PRODUCER REVENUES (Executed-only)</t>
@@ -100,6 +100,27 @@
     <t>Average per Clearing</t>
   </si>
   <si>
+    <t>SOCIAL WELFARE</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Total (EUR)</t>
+  </si>
+  <si>
+    <t>Per Day (EUR)</t>
+  </si>
+  <si>
+    <t>Total Demand Value</t>
+  </si>
+  <si>
+    <t>Total Generation Cost</t>
+  </si>
+  <si>
+    <t>Social Welfare</t>
+  </si>
+  <si>
     <t>GENERATOR PROFITS (Full Revenue - Cost)</t>
   </si>
   <si>
@@ -113,9 +134,6 @@
   </si>
   <si>
     <t>STORAGE REVENUE</t>
-  </si>
-  <si>
-    <t>Metric</t>
   </si>
   <si>
     <t>Per Day</t>
@@ -210,9 +228,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -250,7 +268,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -356,7 +374,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -498,37 +516,37 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C94E993A-79B6-4B85-967C-22D0E13E699D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:E57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF609DF-7FC4-4593-AF5F-428D4CB425A1}">
+  <dimension ref="A1:E63"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -545,112 +563,111 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5">
-        <v>697000.0</v>
+        <v>3665367.2222046107</v>
       </c>
       <c r="C5">
-        <v>6.200981481481482e7</v>
+        <v>342211268.5593155</v>
       </c>
       <c r="D5">
-        <v>88.96673574578884</v>
+        <v>93.363433406130994</v>
       </c>
       <c r="E5">
-        <v>2.066993827160494e6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>11039073.179332757</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6">
-        <v>325072.16644598456</v>
+        <v>1350857.0421643653</v>
       </c>
       <c r="C6">
-        <v>2.9241214558059834e7</v>
+        <v>169800126.84387761</v>
       </c>
       <c r="D6">
-        <v>89.95299375444586</v>
+        <v>125.69807281148053</v>
       </c>
       <c r="E6">
-        <v>974707.1519353278</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>5477423.4465766968</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7">
-        <v>64715.02735472821</v>
+        <v>478445.66307947901</v>
       </c>
       <c r="C7">
-        <v>6.471502735472816e6</v>
+        <v>72231849.461921826</v>
       </c>
       <c r="D7">
-        <v>99.99999999999991</v>
+        <v>150.97189719937481</v>
       </c>
       <c r="E7">
-        <v>215716.75784909388</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>2330059.6600619946</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8">
-        <v>60030.0</v>
+        <v>503486.91100000031</v>
       </c>
       <c r="C8">
-        <v>6.003e6</v>
+        <v>38578750.262571007</v>
       </c>
       <c r="D8">
-        <v>100.0</v>
+        <v>76.623144355327611</v>
       </c>
       <c r="E8">
-        <v>200100.0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>1244475.8149216454</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
         <v>11</v>
       </c>
       <c r="B9">
-        <v>312150.0</v>
+        <v>2887258.772348355</v>
       </c>
       <c r="C9">
-        <v>2.8031838888888884e7</v>
+        <v>137030448.91474897</v>
       </c>
       <c r="D9">
-        <v>89.80246320323205</v>
+        <v>47.460397463194859</v>
       </c>
       <c r="E9">
-        <v>934394.6296296294</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>4420337.0617660955</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
         <v>12</v>
       </c>
       <c r="B10">
-        <v>1.4589671938007127e6</v>
+        <v>8885415.6107968092</v>
       </c>
       <c r="C10">
-        <v>1.3175737099723634e8</v>
-      </c>
-      <c r="D10"/>
+        <v>759852444.04243493</v>
+      </c>
       <c r="E10">
-        <v>4.391912366574544e6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+        <v>24511369.162659191</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -667,110 +684,108 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
         <v>7</v>
       </c>
       <c r="B14">
-        <v>5.640667239652642e7</v>
+        <v>353801679.93586671</v>
       </c>
       <c r="C14">
-        <v>720000.0</v>
+        <v>3803095.8516851799</v>
       </c>
       <c r="D14">
-        <v>720000.0</v>
+        <v>6292927.7061479799</v>
       </c>
       <c r="E14">
-        <v>1.8802224132175473e6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+        <v>11412957.417286023</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
         <v>8</v>
       </c>
       <c r="B15">
-        <v>2.9604285880776655e7</v>
+        <v>213063812.7836518</v>
       </c>
       <c r="C15">
-        <v>335951.6616412533</v>
+        <v>1415113.5920320794</v>
       </c>
       <c r="D15">
-        <v>1.0939910760498121e6</v>
+        <v>4418994.4759038948</v>
       </c>
       <c r="E15">
-        <v>986809.5293592218</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+        <v>6873026.2188274777</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
         <v>9</v>
       </c>
       <c r="B16">
-        <v>1.1063521969490819e7</v>
+        <v>92804879.313542962</v>
       </c>
       <c r="C16">
-        <v>67276.12218312563</v>
+        <v>479750.59997947875</v>
       </c>
       <c r="D16">
-        <v>1.501739340477908e6</v>
+        <v>3142374.8574758656</v>
       </c>
       <c r="E16">
-        <v>368784.06564969395</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+        <v>2993705.7843078375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
         <v>10</v>
       </c>
       <c r="B17">
-        <v>5.489585555555554e6</v>
+        <v>39670596.146329917</v>
       </c>
       <c r="C17">
-        <v>62100.0</v>
+        <v>518474.08800000005</v>
       </c>
       <c r="D17">
-        <v>62100.0</v>
+        <v>518474.08800000005</v>
       </c>
       <c r="E17">
-        <v>182986.18518518514</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
+        <v>1279696.6498816102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
         <v>11</v>
       </c>
       <c r="B18">
-        <v>1.2546795071710816e7</v>
+        <v>-39522450.129126966</v>
       </c>
       <c r="C18">
-        <v>322187.8196059499</v>
+        <v>2945099.6955197365</v>
       </c>
       <c r="D18">
-        <v>2.833463994978871e6</v>
+        <v>15801544.903136302</v>
       </c>
       <c r="E18">
-        <v>418226.5023903605</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
+        <v>-1274917.74610087</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1.1511086087406024e8</v>
-      </c>
-      <c r="C19"/>
-      <c r="D19"/>
+        <v>659818518.05026436</v>
+      </c>
       <c r="E19">
-        <v>3.8370286958020083e6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
+        <v>21284468.324202076</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -781,348 +796,393 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
         <v>7</v>
       </c>
       <c r="B23">
-        <v>2.091e7</v>
+        <v>109961016.66613841</v>
       </c>
       <c r="C23">
-        <v>697000.0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
+        <v>3547129.5698754326</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
         <v>8</v>
       </c>
       <c r="B24">
-        <v>1.950432998675908e7</v>
+        <v>108068563.37314922</v>
       </c>
       <c r="C24">
-        <v>650144.3328919694</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
+        <v>3486082.6894564265</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
         <v>9</v>
       </c>
       <c r="B25">
-        <v>6.471502735472816e6</v>
+        <v>71766849.461921826</v>
       </c>
       <c r="C25">
-        <v>215716.75784909388</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
+        <v>2315059.6600619946</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
         <v>10</v>
       </c>
       <c r="B26">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
         <v>11</v>
       </c>
       <c r="B27">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C27">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
         <v>22</v>
       </c>
       <c r="B28">
-        <v>4.6885832722231895e7</v>
+        <v>289796429.50120944</v>
       </c>
       <c r="C28">
-        <v>1.5628610907410632e6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
+        <v>9348271.9193938524</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
         <v>23</v>
       </c>
       <c r="B29">
-        <v>67171.68011781074</v>
-      </c>
-      <c r="C29"/>
-    </row>
-    <row r="31" spans="1:5">
+        <v>415776.79985826317</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33">
+        <v>2584143745.6844764</v>
+      </c>
+      <c r="C33">
+        <v>83359475.667241171</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34">
+        <v>289796429.50120944</v>
+      </c>
+      <c r="C34">
+        <v>9348271.9193938524</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35">
+        <v>2294347316.1832671</v>
+      </c>
+      <c r="C35">
+        <v>74011203.747847334</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A37" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
         <v>2</v>
       </c>
-      <c r="B32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
+      <c r="B38" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
         <v>7</v>
       </c>
-      <c r="B33">
-        <v>3.549667239652642e7</v>
-      </c>
-      <c r="C33">
-        <v>1.1832224132175473e6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
+      <c r="B39">
+        <v>243840663.2697283</v>
+      </c>
+      <c r="C39">
+        <v>7865827.8474105904</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
         <v>8</v>
       </c>
-      <c r="B34">
-        <v>1.0099955894017573e7</v>
-      </c>
-      <c r="C34">
-        <v>336665.19646725245</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
+      <c r="B40">
+        <v>104995249.41050258</v>
+      </c>
+      <c r="C40">
+        <v>3386943.5293710511</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
         <v>9</v>
       </c>
-      <c r="B35">
-        <v>4.592019234018003e6</v>
-      </c>
-      <c r="C35">
-        <v>153067.3078006001</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" t="s">
+      <c r="B41">
+        <v>21038029.851621136</v>
+      </c>
+      <c r="C41">
+        <v>678646.12424584315</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
         <v>10</v>
       </c>
-      <c r="B36">
-        <v>5.489585555555554e6</v>
-      </c>
-      <c r="C36">
-        <v>182986.18518518514</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" t="s">
+      <c r="B42">
+        <v>39670596.146329917</v>
+      </c>
+      <c r="C42">
+        <v>1279696.6498816102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
         <v>11</v>
       </c>
-      <c r="B37">
-        <v>1.2546795071710816e7</v>
-      </c>
-      <c r="C37">
-        <v>418226.5023903605</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38">
-        <v>6.822502815182836e7</v>
-      </c>
-      <c r="C38">
-        <v>2.2741676050609457e6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" t="s">
-        <v>29</v>
-      </c>
-      <c r="B41" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42">
-        <v>19100.858096999476</v>
-      </c>
-      <c r="C42">
-        <v>636.6952698999826</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>32</v>
-      </c>
       <c r="B43">
-        <v>23646.472989460806</v>
+        <v>-39522450.129126966</v>
       </c>
       <c r="C43">
-        <v>788.2157663153602</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
+        <v>-1274917.74610087</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A44" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B44">
-        <v>99.5894347552996</v>
-      </c>
-      <c r="C44"/>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" t="s">
-        <v>34</v>
-      </c>
-      <c r="B45">
-        <v>67.54834677465387</v>
-      </c>
-      <c r="C45"/>
-    </row>
-    <row r="46" spans="1:5">
+        <v>370022088.54905498</v>
+      </c>
+      <c r="C44">
+        <v>11936196.404808227</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A46" t="s">
         <v>35</v>
       </c>
-      <c r="B46">
-        <v>1.9022436612213657e6</v>
-      </c>
-      <c r="C46">
-        <v>63408.12204071219</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" t="s">
         <v>36</v>
       </c>
-      <c r="B47">
-        <v>1.5972801574895845e6</v>
-      </c>
-      <c r="C47">
-        <v>53242.67191631949</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5">
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A48" t="s">
         <v>37</v>
       </c>
       <c r="B48">
-        <v>304963.50373178115</v>
+        <v>166466.90616790851</v>
       </c>
       <c r="C48">
-        <v>10165.450124392704</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
+        <v>5369.9001989647904</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
         <v>38</v>
       </c>
       <c r="B49">
-        <v>436.9104637991134</v>
-      </c>
-      <c r="C49"/>
-    </row>
-    <row r="51" spans="1:5">
+        <v>167983.83477519566</v>
+      </c>
+      <c r="C49">
+        <v>5418.8333798450212</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50">
+        <v>86.756124727944837</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A51" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5">
+        <v>40</v>
+      </c>
+      <c r="B51">
+        <v>53.479018094525657</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A52" t="s">
+        <v>41</v>
+      </c>
+      <c r="B52">
+        <v>14442023.67457816</v>
+      </c>
+      <c r="C52">
+        <v>465871.73143800517</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
+        <v>42</v>
+      </c>
+      <c r="B53">
+        <v>8983610.539530497</v>
+      </c>
+      <c r="C53">
+        <v>289793.88837195153</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
+        <v>43</v>
+      </c>
+      <c r="B54">
+        <v>5458413.135047663</v>
+      </c>
+      <c r="C54">
+        <v>176077.84306605364</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
+        <v>44</v>
+      </c>
+      <c r="B55">
+        <v>7831.2957461229025</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
         <v>2</v>
       </c>
-      <c r="B52" t="s">
-        <v>40</v>
-      </c>
-      <c r="C52" t="s">
-        <v>41</v>
-      </c>
-      <c r="D52" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" t="s">
+      <c r="B58" t="s">
+        <v>46</v>
+      </c>
+      <c r="C58" t="s">
+        <v>47</v>
+      </c>
+      <c r="D58" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
         <v>7</v>
       </c>
-      <c r="B53">
-        <v>697000.0</v>
-      </c>
-      <c r="C53">
-        <v>697000.0</v>
-      </c>
-      <c r="D53">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" t="s">
+      <c r="B59">
+        <v>3665367.2222046107</v>
+      </c>
+      <c r="C59">
+        <v>3665367.2222046107</v>
+      </c>
+      <c r="D59">
+        <v>4.5474735088646412E-13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
         <v>8</v>
       </c>
-      <c r="B54">
-        <v>325072.16644598456</v>
-      </c>
-      <c r="C54">
-        <v>325072.16644598456</v>
-      </c>
-      <c r="D54">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="A55" t="s">
+      <c r="B60">
+        <v>1350857.0421643653</v>
+      </c>
+      <c r="C60">
+        <v>1350857.0421643653</v>
+      </c>
+      <c r="D60">
+        <v>4.5474735088646412E-13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
         <v>9</v>
       </c>
-      <c r="B55">
-        <v>64715.02735472821</v>
-      </c>
-      <c r="C55">
-        <v>64715.02735472821</v>
-      </c>
-      <c r="D55">
-        <v>5.684341886080802e-14</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5">
-      <c r="A56" t="s">
+      <c r="B61">
+        <v>478445.66307947901</v>
+      </c>
+      <c r="C61">
+        <v>478445.66307947901</v>
+      </c>
+      <c r="D61">
+        <v>9.0949470177292824E-13</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
         <v>10</v>
       </c>
-      <c r="B56">
-        <v>60030.0</v>
-      </c>
-      <c r="C56">
-        <v>60030.0</v>
-      </c>
-      <c r="D56">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="A57" t="s">
+      <c r="B62">
+        <v>503486.91100000031</v>
+      </c>
+      <c r="C62">
+        <v>503486.91100000031</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
         <v>11</v>
       </c>
-      <c r="B57">
-        <v>312150.0</v>
-      </c>
-      <c r="C57">
-        <v>312150.0</v>
-      </c>
-      <c r="D57">
-        <v>2.2737367544323206e-13</v>
+      <c r="B63">
+        <v>2887258.772348355</v>
+      </c>
+      <c r="C63">
+        <v>2887258.772348355</v>
+      </c>
+      <c r="D63">
+        <v>1.8189894035458565E-12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added wind samples, daily analysis and drivers
</commit_message>
<xml_diff>
--- a/market_clearing/economic_summary.xlsx
+++ b/market_clearing/economic_summary.xlsx
@@ -1,43 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10513"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/laura_linuesa-domenech_tennet_eu/Documents/Thesis/Code/market_clearing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipenoris/tmp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="115_{EA2E6AE5-D56F-45D1-9A47-0899E809A698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D507512-55AE-4F7F-8EB4-559EC3C6DCF6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C353BCB8-5EC8-0143-BDD3-A1B661DAACD7}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7260" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="380" yWindow="460" windowWidth="28040" windowHeight="17040" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" r:id="rId4" sheetId="2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="53">
   <si>
     <t>ECONOMIC SUMMARY (30 days simulation)</t>
   </si>
@@ -202,18 +191,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -239,16 +217,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -264,14 +239,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -309,7 +280,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -415,7 +386,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -557,705 +528,706 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{723E3204-9272-4F57-AC54-4C74800A6B0B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87F505F2-E667-4F42-9764-E694A6C2A40A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
   <dimension ref="A1:F64"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
-  <cols>
-    <col min="2" max="3" width="15.9375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.3125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.4375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.0625" style="1" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="1">
-        <v>108.76824513184334</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="F4">
+        <v>34.94128195357986</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
-        <v>2811043012.3559942</v>
-      </c>
-      <c r="C5" s="1">
-        <v>93701433.745199814</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="B5">
+        <v>2.363858574078856e9</v>
+      </c>
+      <c r="C5">
+        <v>7.879528580262853e7</v>
+      </c>
+      <c r="E5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="1">
-        <v>18892.793002505448</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="F5">
+        <v>477425.89021656604</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1">
-        <v>359629075.69536591</v>
-      </c>
-      <c r="C6" s="1">
-        <v>11987635.856512196</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B6">
+        <v>9.038016991960563e7</v>
+      </c>
+      <c r="C6">
+        <v>3.0126723306535208e6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="1">
-        <v>2451413936.6606283</v>
-      </c>
-      <c r="C7" s="1">
-        <v>81713797.888687611</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B7">
+        <v>2.2734784041592503e9</v>
+      </c>
+      <c r="C7">
+        <v>7.578261347197501e7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="1">
-        <v>3982876.9199949773</v>
-      </c>
-      <c r="C11" s="1">
-        <v>445596795.14286435</v>
-      </c>
-      <c r="D11" s="1">
-        <v>111.87812329973437</v>
-      </c>
-      <c r="E11" s="1">
-        <v>14853226.504762145</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B11">
+        <v>2.441670279609822e6</v>
+      </c>
+      <c r="C11">
+        <v>1.4421625352984518e8</v>
+      </c>
+      <c r="D11">
+        <v>59.06458981549748</v>
+      </c>
+      <c r="E11">
+        <v>4.807208450994839e6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="1">
-        <v>1628038.5824713197</v>
-      </c>
-      <c r="C12" s="1">
-        <v>236128137.90835813</v>
-      </c>
-      <c r="D12" s="1">
-        <v>145.03841644214711</v>
-      </c>
-      <c r="E12" s="1">
-        <v>7870937.9302786039</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B12">
+        <v>209105.80709560722</v>
+      </c>
+      <c r="C12">
+        <v>1.7941127300796688e7</v>
+      </c>
+      <c r="D12">
+        <v>85.79927812618641</v>
+      </c>
+      <c r="E12">
+        <v>598037.576693223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="1">
-        <v>732664.54331873974</v>
-      </c>
-      <c r="C13" s="1">
-        <v>134703014.83114436</v>
-      </c>
-      <c r="D13" s="1">
-        <v>183.85360129614313</v>
-      </c>
-      <c r="E13" s="1">
-        <v>4490100.4943714784</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B13">
+        <v>2677.313091082088</v>
+      </c>
+      <c r="C13">
+        <v>401596.9636623132</v>
+      </c>
+      <c r="D13">
+        <v>150.0</v>
+      </c>
+      <c r="E13">
+        <v>13386.565455410439</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="1">
-        <v>478312.56544999999</v>
-      </c>
-      <c r="C14" s="1">
-        <v>38925180.534927145</v>
-      </c>
-      <c r="D14" s="1">
-        <v>81.380217344501602</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1297506.0178309048</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B14">
+        <v>3.3456774043698427e6</v>
+      </c>
+      <c r="C14">
+        <v>4.228518862998185e7</v>
+      </c>
+      <c r="D14">
+        <v>12.638752491424455</v>
+      </c>
+      <c r="E14">
+        <v>1.4095062876660617e6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="1">
-        <v>2763928.8547474938</v>
-      </c>
-      <c r="C15" s="1">
-        <v>187279850.58477989</v>
-      </c>
-      <c r="D15" s="1">
-        <v>67.758564140714597</v>
-      </c>
-      <c r="E15" s="1">
-        <v>6242661.6861593295</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="B15">
+        <v>2.4061535773834353e6</v>
+      </c>
+      <c r="C15">
+        <v>8.884724505146629e7</v>
+      </c>
+      <c r="D15">
+        <v>36.92501006028176</v>
+      </c>
+      <c r="E15">
+        <v>2.9615748350488762e6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="1">
-        <v>9585821.4659825303</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1042632979.0020738</v>
-      </c>
-      <c r="E16" s="1">
-        <v>34754432.633402459</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B16">
+        <v>8.40528438154979e6</v>
+      </c>
+      <c r="C16">
+        <v>2.9369141147575235e8</v>
+      </c>
+      <c r="D16"/>
+      <c r="E16">
+        <v>9.789713715858411e6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="1">
-        <v>448566332.41025943</v>
-      </c>
-      <c r="C20" s="1">
-        <v>4120876.9199949773</v>
-      </c>
-      <c r="D20" s="1">
-        <v>4634643.3879737807</v>
-      </c>
-      <c r="E20" s="1">
-        <v>14952211.080341982</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B20">
+        <v>1.3437437947017145e8</v>
+      </c>
+      <c r="C20">
+        <v>2.5902230518127065e6</v>
+      </c>
+      <c r="D20">
+        <v>5.164434124776814e6</v>
+      </c>
+      <c r="E20">
+        <v>4.479145982339049e6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="1">
-        <v>243394966.75958812</v>
-      </c>
-      <c r="C21" s="1">
-        <v>1717754.4742361107</v>
-      </c>
-      <c r="D21" s="1">
-        <v>2652099.8573610727</v>
-      </c>
-      <c r="E21" s="1">
-        <v>8113165.5586529374</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B21">
+        <v>2.191522176791359e7</v>
+      </c>
+      <c r="C21">
+        <v>243412.3356109523</v>
+      </c>
+      <c r="D21">
+        <v>3.0366617333832057e6</v>
+      </c>
+      <c r="E21">
+        <v>730507.3922637864</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="1">
-        <v>137343384.36182228</v>
-      </c>
-      <c r="C22" s="1">
-        <v>761478.05516458466</v>
-      </c>
-      <c r="D22" s="1">
-        <v>2061822.8216769036</v>
-      </c>
-      <c r="E22" s="1">
-        <v>4578112.8120607426</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B22">
+        <v>401596.9636623132</v>
+      </c>
+      <c r="C22">
+        <v>2677.313091082088</v>
+      </c>
+      <c r="D22">
+        <v>6681.902858463811</v>
+      </c>
+      <c r="E22">
+        <v>13386.565455410439</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="1">
-        <v>40159749.943126753</v>
-      </c>
-      <c r="C23" s="1">
-        <v>492550.3836</v>
-      </c>
-      <c r="D23" s="1">
-        <v>492550.3836</v>
-      </c>
-      <c r="E23" s="1">
-        <v>1338658.3314375584</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B23">
+        <v>2.8935137205064368e7</v>
+      </c>
+      <c r="C23">
+        <v>3.5114889423198453e6</v>
+      </c>
+      <c r="D23">
+        <v>3.633866564613981e6</v>
+      </c>
+      <c r="E23">
+        <v>964504.5735021456</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="1">
-        <v>169561145.75714132</v>
-      </c>
-      <c r="C24" s="1">
-        <v>2808100.0982027063</v>
-      </c>
-      <c r="D24" s="1">
-        <v>5131115.2235797457</v>
-      </c>
-      <c r="E24" s="1">
-        <v>5652038.1919047106</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B24">
+        <v>5.942600162206786e7</v>
+      </c>
+      <c r="C24">
+        <v>2.439377909690926e6</v>
+      </c>
+      <c r="D24">
+        <v>8.414383402899928e6</v>
+      </c>
+      <c r="E24">
+        <v>1.9808667207355953e6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="1">
-        <v>1039025579.2319379</v>
-      </c>
-      <c r="E25" s="1">
-        <v>34634185.974397928</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B25">
+        <v>2.4505233702887958e8</v>
+      </c>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25">
+        <v>8.168411234295986e6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="1">
-        <v>119486307.59984931</v>
-      </c>
-      <c r="C29" s="1">
-        <v>3982876.9199949773</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B29">
+        <v>7.325010838829473e7</v>
+      </c>
+      <c r="C29">
+        <v>2.441670279609824e6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="1">
-        <v>130243086.59770559</v>
-      </c>
-      <c r="C30" s="1">
-        <v>4341436.2199235195</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B30">
+        <v>1.6728464567648584e7</v>
+      </c>
+      <c r="C30">
+        <v>557615.4855882862</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="1">
-        <v>109899681.497811</v>
-      </c>
-      <c r="C31" s="1">
-        <v>3663322.7165937</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="B31">
+        <v>401596.9636623132</v>
+      </c>
+      <c r="C31">
+        <v>13386.565455410439</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="1">
-        <v>0</v>
-      </c>
-      <c r="C32" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B32">
+        <v>0.0</v>
+      </c>
+      <c r="C32">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="1">
-        <v>0</v>
-      </c>
-      <c r="C33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B33">
+        <v>0.0</v>
+      </c>
+      <c r="C33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="1">
-        <v>359629075.69536591</v>
-      </c>
-      <c r="C34" s="1">
-        <v>11987635.856512196</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B34">
+        <v>9.038016991960563e7</v>
+      </c>
+      <c r="C34">
+        <v>3.0126723306535208e6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="1">
-        <v>515967.11003639299</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B35">
+        <v>129670.25813429788</v>
+      </c>
+      <c r="C35"/>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>35</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="1">
-        <v>329080024.81041014</v>
-      </c>
-      <c r="C39" s="1">
-        <v>10969334.160347005</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B39">
+        <v>6.1124271081876725e7</v>
+      </c>
+      <c r="C39">
+        <v>2.0374757027292242e6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>18</v>
       </c>
-      <c r="B40" s="1">
-        <v>113151880.16188253</v>
-      </c>
-      <c r="C40" s="1">
-        <v>3771729.3387294179</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B40">
+        <v>5.186757200265007e6</v>
+      </c>
+      <c r="C40">
+        <v>172891.90667550024</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="1">
-        <v>27443702.864011273</v>
-      </c>
-      <c r="C41" s="1">
-        <v>914790.09546704241</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B41">
+        <v>0.0</v>
+      </c>
+      <c r="C41">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="1">
-        <v>40159749.943126753</v>
-      </c>
-      <c r="C42" s="1">
-        <v>1338658.3314375584</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B42">
+        <v>2.8935137205064368e7</v>
+      </c>
+      <c r="C42">
+        <v>964504.5735021456</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>21</v>
       </c>
-      <c r="B43" s="1">
-        <v>169561145.75714132</v>
-      </c>
-      <c r="C43" s="1">
-        <v>5652038.1919047106</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B43">
+        <v>5.942600162206786e7</v>
+      </c>
+      <c r="C43">
+        <v>1.9808667207355953e6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>37</v>
       </c>
-      <c r="B44" s="1">
-        <v>679396503.53657198</v>
-      </c>
-      <c r="C44" s="1">
-        <v>22646550.117885731</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="B44">
+        <v>1.5467216710927397e8</v>
+      </c>
+      <c r="C44">
+        <v>5.155738903642465e6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>22</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>40</v>
       </c>
-      <c r="B48" s="1">
-        <v>204599.28922255122</v>
-      </c>
-      <c r="C48" s="1">
-        <v>6819.9763074183738</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B48">
+        <v>186646.16972543</v>
+      </c>
+      <c r="C48">
+        <v>6221.538990847666</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>41</v>
       </c>
-      <c r="B49" s="1">
-        <v>253251.40078956936</v>
-      </c>
-      <c r="C49" s="1">
-        <v>8441.7133596523126</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B49">
+        <v>235094.03669806186</v>
+      </c>
+      <c r="C49">
+        <v>7836.467889935395</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="1">
-        <v>147.37183863930306</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B50">
+        <v>69.23345012601534</v>
+      </c>
+      <c r="C50"/>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>43</v>
       </c>
-      <c r="B51" s="1">
-        <v>82.831418924411182</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B51">
+        <v>12.621227828932595</v>
+      </c>
+      <c r="C51"/>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>44</v>
       </c>
-      <c r="B52" s="1">
-        <v>30152173.437021919</v>
-      </c>
-      <c r="C52" s="1">
-        <v>1005072.4479007307</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B52">
+        <v>1.2922158282897351e7</v>
+      </c>
+      <c r="C52">
+        <v>430738.6094299117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>45</v>
       </c>
-      <c r="B53" s="1">
-        <v>20977172.871994779</v>
-      </c>
-      <c r="C53" s="1">
-        <v>699239.09573315934</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B53">
+        <v>2.967175398389679e6</v>
+      </c>
+      <c r="C53">
+        <v>98905.84661298929</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
       <c r="A54" t="s">
         <v>46</v>
       </c>
-      <c r="B54" s="1">
-        <v>9175000.5650271401</v>
-      </c>
-      <c r="C54" s="1">
-        <v>305833.35216757131</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B54">
+        <v>9.954982884507673e6</v>
+      </c>
+      <c r="C54">
+        <v>331832.76281692245</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
       <c r="A55" t="s">
         <v>47</v>
       </c>
-      <c r="B55" s="1">
-        <v>48058.394437018149</v>
-      </c>
-      <c r="C55" s="1">
-        <v>1601.9464812339384</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B55">
+        <v>44247.86697263186</v>
+      </c>
+      <c r="C55">
+        <v>1474.9288990877287</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
       <c r="A56" t="s">
         <v>48</v>
       </c>
-      <c r="B56" s="1">
-        <v>593.71712999999988</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B56">
+        <v>4200.0</v>
+      </c>
+      <c r="C56"/>
+    </row>
+    <row r="58" spans="1:6">
       <c r="A58" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="59" spans="1:6">
       <c r="A59" t="s">
         <v>12</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>50</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" t="s">
         <v>51</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D59" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="60" spans="1:6">
       <c r="A60" t="s">
         <v>17</v>
       </c>
-      <c r="B60" s="1">
-        <v>3982876.9199949773</v>
-      </c>
-      <c r="C60" s="1">
-        <v>3982876.9199949773</v>
-      </c>
-      <c r="D60" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B60">
+        <v>2.441670279609822e6</v>
+      </c>
+      <c r="C60">
+        <v>2.441670279609822e6</v>
+      </c>
+      <c r="D60">
+        <v>2.842170943040401e-14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
       <c r="A61" t="s">
         <v>18</v>
       </c>
-      <c r="B61" s="1">
-        <v>1628038.5824713197</v>
-      </c>
-      <c r="C61" s="1">
-        <v>1628038.5824713197</v>
-      </c>
-      <c r="D61" s="1">
-        <v>1.1368683772161603E-13</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B61">
+        <v>209105.80709560722</v>
+      </c>
+      <c r="C61">
+        <v>209105.80709560722</v>
+      </c>
+      <c r="D61">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
       <c r="A62" t="s">
         <v>19</v>
       </c>
-      <c r="B62" s="1">
-        <v>732664.54331873974</v>
-      </c>
-      <c r="C62" s="1">
-        <v>732664.54331873974</v>
-      </c>
-      <c r="D62" s="1">
-        <v>4.5474735088646412E-13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B62">
+        <v>2677.313091082088</v>
+      </c>
+      <c r="C62">
+        <v>2677.313091082088</v>
+      </c>
+      <c r="D62">
+        <v>7.105427357601002e-15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63" t="s">
         <v>20</v>
       </c>
-      <c r="B63" s="1">
-        <v>478312.56544999999</v>
-      </c>
-      <c r="C63" s="1">
-        <v>478312.56544999999</v>
-      </c>
-      <c r="D63" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B63">
+        <v>3.3456774043698427e6</v>
+      </c>
+      <c r="C63">
+        <v>3.3456774043698427e6</v>
+      </c>
+      <c r="D63">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
       <c r="A64" t="s">
         <v>21</v>
       </c>
-      <c r="B64" s="1">
-        <v>2763928.8547474938</v>
-      </c>
-      <c r="C64" s="1">
-        <v>2763928.8547474938</v>
-      </c>
-      <c r="D64" s="1">
-        <v>0</v>
+      <c r="B64">
+        <v>2.4061535773834353e6</v>
+      </c>
+      <c r="C64">
+        <v>2.4061535773834353e6</v>
+      </c>
+      <c r="D64">
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>